<commit_message>
mis cambios en rama dev
</commit_message>
<xml_diff>
--- a/sealand/CheckListSealand.xlsx
+++ b/sealand/CheckListSealand.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karinabanda/Desktop/Proyectos/Reportes/Reportes Diarios/Sealend/proyecto/seland/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karinabanda/Desktop/Proyectos/Reportes/Reportes Diarios/Sealend/proyecto/sealand/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE0D657-942C-764E-B6AA-BBD94825AE6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52CCBD55-6ADD-5043-855D-B625E54BD192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
   <si>
     <t>CPU Utilization Last Hour</t>
   </si>
@@ -67,9 +67,6 @@
   </si>
   <si>
     <t>Disponibilidad de la URL / Página web</t>
-  </si>
-  <si>
-    <t>Free Storages Space Last Hour</t>
   </si>
   <si>
     <t>La revisión realizada se basa en los siguientes criterios:
@@ -200,7 +197,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -484,24 +481,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -516,10 +500,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -533,114 +513,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -649,6 +521,111 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -894,65 +871,57 @@
   <sheetData>
     <row r="1" spans="2:21" ht="15.75" customHeight="1"/>
     <row r="2" spans="2:21" ht="27" customHeight="1">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
-      <c r="L2" s="47"/>
-      <c r="M2" s="47"/>
-      <c r="O2" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="P2" s="41"/>
-      <c r="Q2" s="41"/>
-      <c r="R2" s="41"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
+      <c r="O2" s="45" t="s">
+        <v>19</v>
+      </c>
+      <c r="P2" s="46"/>
+      <c r="Q2" s="46"/>
+      <c r="R2" s="46"/>
     </row>
     <row r="3" spans="2:21" ht="27" customHeight="1">
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="38"/>
-      <c r="E3" s="39"/>
-      <c r="F3" s="19" t="s">
+      <c r="D3" s="49"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="38"/>
-      <c r="H3" s="39"/>
-      <c r="I3" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="J3" s="38"/>
-      <c r="K3" s="42"/>
-      <c r="L3" s="43" t="s">
+      <c r="G3" s="49"/>
+      <c r="H3" s="50"/>
+      <c r="I3" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="M3" s="44"/>
-      <c r="O3" s="24" t="s">
+      <c r="J3" s="52"/>
+      <c r="O3" s="43" t="s">
+        <v>15</v>
+      </c>
+      <c r="P3" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="P3" s="24" t="s">
+      <c r="Q3" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="Q3" s="24" t="s">
+      <c r="R3" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="R3" s="24" t="s">
-        <v>19</v>
-      </c>
     </row>
     <row r="4" spans="2:21" ht="22" customHeight="1">
-      <c r="B4" s="40"/>
+      <c r="B4" s="44"/>
       <c r="C4" s="2" t="s">
         <v>1</v>
       </c>
@@ -971,21 +940,12 @@
       <c r="H4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="K4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="L4" s="45"/>
-      <c r="M4" s="46"/>
-      <c r="O4" s="40"/>
-      <c r="P4" s="40"/>
-      <c r="Q4" s="40"/>
-      <c r="R4" s="40"/>
+      <c r="I4" s="53"/>
+      <c r="J4" s="54"/>
+      <c r="O4" s="44"/>
+      <c r="P4" s="44"/>
+      <c r="Q4" s="44"/>
+      <c r="R4" s="44"/>
     </row>
     <row r="5" spans="2:21" ht="15.75" customHeight="1">
       <c r="B5" s="1"/>
@@ -995,11 +955,8 @@
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="17"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="15"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
@@ -1016,26 +973,26 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
-      <c r="S7" s="13"/>
-      <c r="T7" s="13"/>
-      <c r="U7" s="12"/>
+      <c r="S7" s="11"/>
+      <c r="T7" s="11"/>
+      <c r="U7" s="10"/>
     </row>
     <row r="8" spans="2:21" ht="22" customHeight="1">
-      <c r="B8" s="54" t="s">
+      <c r="B8" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="54"/>
-      <c r="D8" s="54"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="54"/>
-      <c r="H8" s="51" t="s">
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="H8" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="I8" s="52"/>
-      <c r="J8" s="52"/>
-      <c r="K8" s="52"/>
-      <c r="L8" s="52"/>
-      <c r="M8" s="53"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="23"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
@@ -1047,16 +1004,16 @@
       <c r="D9" s="8"/>
       <c r="E9" s="8"/>
       <c r="F9" s="9"/>
-      <c r="H9" s="56"/>
-      <c r="I9" s="57"/>
-      <c r="J9" s="57"/>
-      <c r="K9" s="57"/>
-      <c r="L9" s="57"/>
-      <c r="M9" s="58"/>
-      <c r="O9" s="55"/>
-      <c r="P9" s="55"/>
-      <c r="Q9" s="55"/>
-      <c r="R9" s="55"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="20"/>
+      <c r="O9" s="17"/>
+      <c r="P9" s="17"/>
+      <c r="Q9" s="17"/>
+      <c r="R9" s="17"/>
     </row>
     <row r="10" spans="2:21" ht="15.75" customHeight="1">
       <c r="O10" s="5"/>
@@ -1071,12 +1028,12 @@
       <c r="R11" s="5"/>
     </row>
     <row r="12" spans="2:21" ht="23" customHeight="1">
-      <c r="B12" s="48" t="s">
+      <c r="B12" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="49"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="50"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="42"/>
       <c r="O12" s="5"/>
       <c r="P12" s="5"/>
       <c r="Q12" s="5"/>
@@ -1129,7 +1086,7 @@
       <c r="P16" s="5"/>
       <c r="Q16" s="5"/>
       <c r="R16" s="5"/>
-      <c r="U16" s="13"/>
+      <c r="U16" s="11"/>
     </row>
     <row r="17" spans="2:21" ht="15.75" customHeight="1">
       <c r="B17" s="6"/>
@@ -1140,7 +1097,7 @@
       <c r="P17" s="5"/>
       <c r="Q17" s="5"/>
       <c r="R17" s="5"/>
-      <c r="U17" s="13"/>
+      <c r="U17" s="11"/>
     </row>
     <row r="18" spans="2:21" ht="15.75" customHeight="1">
       <c r="B18" s="6"/>
@@ -1155,164 +1112,164 @@
       <c r="E19" s="5"/>
     </row>
     <row r="20" spans="2:21" ht="24" customHeight="1">
-      <c r="G20" s="34" t="s">
+      <c r="G20" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="H20" s="35"/>
-      <c r="I20" s="35"/>
-      <c r="J20" s="35"/>
-      <c r="K20" s="35"/>
-      <c r="L20" s="35"/>
-      <c r="M20" s="36"/>
+      <c r="H20" s="25"/>
+      <c r="I20" s="25"/>
+      <c r="J20" s="25"/>
+      <c r="K20" s="25"/>
+      <c r="L20" s="25"/>
+      <c r="M20" s="26"/>
     </row>
     <row r="21" spans="2:21" ht="15.75" customHeight="1">
-      <c r="G21" s="20"/>
-      <c r="H21" s="21"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="21"/>
-      <c r="L21" s="21"/>
-      <c r="M21" s="22"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="28"/>
+      <c r="I21" s="28"/>
+      <c r="J21" s="28"/>
+      <c r="K21" s="28"/>
+      <c r="L21" s="28"/>
+      <c r="M21" s="29"/>
     </row>
     <row r="22" spans="2:21" ht="15.75" customHeight="1">
-      <c r="G22" s="20"/>
-      <c r="H22" s="21"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="21"/>
-      <c r="L22" s="21"/>
-      <c r="M22" s="22"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="28"/>
+      <c r="I22" s="28"/>
+      <c r="J22" s="28"/>
+      <c r="K22" s="28"/>
+      <c r="L22" s="28"/>
+      <c r="M22" s="29"/>
     </row>
     <row r="23" spans="2:21" ht="15" customHeight="1">
-      <c r="G23" s="20"/>
-      <c r="H23" s="21"/>
-      <c r="I23" s="21"/>
-      <c r="J23" s="21"/>
-      <c r="K23" s="21"/>
-      <c r="L23" s="21"/>
-      <c r="M23" s="22"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="28"/>
+      <c r="I23" s="28"/>
+      <c r="J23" s="28"/>
+      <c r="K23" s="28"/>
+      <c r="L23" s="28"/>
+      <c r="M23" s="29"/>
     </row>
     <row r="25" spans="2:21" ht="17" customHeight="1"/>
     <row r="26" spans="2:21" ht="24" customHeight="1">
-      <c r="G26" s="14" t="s">
+      <c r="G26" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="H26" s="15"/>
-      <c r="I26" s="15"/>
-      <c r="J26" s="15"/>
-      <c r="K26" s="15"/>
-      <c r="L26" s="15"/>
-      <c r="M26" s="16"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
+      <c r="L26" s="13"/>
+      <c r="M26" s="14"/>
     </row>
     <row r="27" spans="2:21" ht="15.75" customHeight="1">
-      <c r="G27" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="H27" s="26"/>
-      <c r="I27" s="26"/>
-      <c r="J27" s="26"/>
-      <c r="K27" s="26"/>
-      <c r="L27" s="26"/>
-      <c r="M27" s="27"/>
+      <c r="G27" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="32"/>
+      <c r="L27" s="32"/>
+      <c r="M27" s="33"/>
     </row>
     <row r="28" spans="2:21" ht="15.75" customHeight="1">
-      <c r="G28" s="28"/>
-      <c r="H28" s="37"/>
-      <c r="I28" s="37"/>
-      <c r="J28" s="37"/>
-      <c r="K28" s="37"/>
-      <c r="L28" s="37"/>
-      <c r="M28" s="29"/>
+      <c r="G28" s="34"/>
+      <c r="H28" s="35"/>
+      <c r="I28" s="35"/>
+      <c r="J28" s="35"/>
+      <c r="K28" s="35"/>
+      <c r="L28" s="35"/>
+      <c r="M28" s="36"/>
     </row>
     <row r="29" spans="2:21" ht="15" customHeight="1">
-      <c r="G29" s="28"/>
-      <c r="H29" s="37"/>
-      <c r="I29" s="37"/>
-      <c r="J29" s="37"/>
-      <c r="K29" s="37"/>
-      <c r="L29" s="37"/>
-      <c r="M29" s="29"/>
+      <c r="G29" s="34"/>
+      <c r="H29" s="35"/>
+      <c r="I29" s="35"/>
+      <c r="J29" s="35"/>
+      <c r="K29" s="35"/>
+      <c r="L29" s="35"/>
+      <c r="M29" s="36"/>
     </row>
     <row r="30" spans="2:21" ht="15.75" customHeight="1">
-      <c r="G30" s="28"/>
-      <c r="H30" s="37"/>
-      <c r="I30" s="37"/>
-      <c r="J30" s="37"/>
-      <c r="K30" s="37"/>
-      <c r="L30" s="37"/>
-      <c r="M30" s="29"/>
+      <c r="G30" s="34"/>
+      <c r="H30" s="35"/>
+      <c r="I30" s="35"/>
+      <c r="J30" s="35"/>
+      <c r="K30" s="35"/>
+      <c r="L30" s="35"/>
+      <c r="M30" s="36"/>
     </row>
     <row r="31" spans="2:21" ht="15.75" customHeight="1">
-      <c r="G31" s="28"/>
-      <c r="H31" s="37"/>
-      <c r="I31" s="37"/>
-      <c r="J31" s="37"/>
-      <c r="K31" s="37"/>
-      <c r="L31" s="37"/>
-      <c r="M31" s="29"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="35"/>
+      <c r="I31" s="35"/>
+      <c r="J31" s="35"/>
+      <c r="K31" s="35"/>
+      <c r="L31" s="35"/>
+      <c r="M31" s="36"/>
     </row>
     <row r="32" spans="2:21" ht="15.75" customHeight="1">
-      <c r="G32" s="28"/>
-      <c r="H32" s="37"/>
-      <c r="I32" s="37"/>
-      <c r="J32" s="37"/>
-      <c r="K32" s="37"/>
-      <c r="L32" s="37"/>
-      <c r="M32" s="29"/>
+      <c r="G32" s="34"/>
+      <c r="H32" s="35"/>
+      <c r="I32" s="35"/>
+      <c r="J32" s="35"/>
+      <c r="K32" s="35"/>
+      <c r="L32" s="35"/>
+      <c r="M32" s="36"/>
     </row>
     <row r="33" spans="7:13" ht="15.75" customHeight="1">
-      <c r="G33" s="28"/>
-      <c r="H33" s="37"/>
-      <c r="I33" s="37"/>
-      <c r="J33" s="37"/>
-      <c r="K33" s="37"/>
-      <c r="L33" s="37"/>
-      <c r="M33" s="29"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="35"/>
+      <c r="I33" s="35"/>
+      <c r="J33" s="35"/>
+      <c r="K33" s="35"/>
+      <c r="L33" s="35"/>
+      <c r="M33" s="36"/>
     </row>
     <row r="34" spans="7:13" ht="15.75" customHeight="1">
-      <c r="G34" s="28"/>
-      <c r="H34" s="37"/>
-      <c r="I34" s="37"/>
-      <c r="J34" s="37"/>
-      <c r="K34" s="37"/>
-      <c r="L34" s="37"/>
-      <c r="M34" s="29"/>
+      <c r="G34" s="34"/>
+      <c r="H34" s="35"/>
+      <c r="I34" s="35"/>
+      <c r="J34" s="35"/>
+      <c r="K34" s="35"/>
+      <c r="L34" s="35"/>
+      <c r="M34" s="36"/>
     </row>
     <row r="35" spans="7:13" ht="15.75" customHeight="1">
-      <c r="G35" s="28"/>
-      <c r="H35" s="37"/>
-      <c r="I35" s="37"/>
-      <c r="J35" s="37"/>
-      <c r="K35" s="37"/>
-      <c r="L35" s="37"/>
-      <c r="M35" s="29"/>
+      <c r="G35" s="34"/>
+      <c r="H35" s="35"/>
+      <c r="I35" s="35"/>
+      <c r="J35" s="35"/>
+      <c r="K35" s="35"/>
+      <c r="L35" s="35"/>
+      <c r="M35" s="36"/>
     </row>
     <row r="36" spans="7:13" ht="15.75" customHeight="1">
-      <c r="G36" s="28"/>
-      <c r="H36" s="37"/>
-      <c r="I36" s="37"/>
-      <c r="J36" s="37"/>
-      <c r="K36" s="37"/>
-      <c r="L36" s="37"/>
-      <c r="M36" s="29"/>
+      <c r="G36" s="34"/>
+      <c r="H36" s="35"/>
+      <c r="I36" s="35"/>
+      <c r="J36" s="35"/>
+      <c r="K36" s="35"/>
+      <c r="L36" s="35"/>
+      <c r="M36" s="36"/>
     </row>
     <row r="37" spans="7:13" ht="15.75" customHeight="1">
-      <c r="G37" s="28"/>
-      <c r="H37" s="37"/>
-      <c r="I37" s="37"/>
-      <c r="J37" s="37"/>
-      <c r="K37" s="37"/>
-      <c r="L37" s="37"/>
-      <c r="M37" s="29"/>
+      <c r="G37" s="34"/>
+      <c r="H37" s="35"/>
+      <c r="I37" s="35"/>
+      <c r="J37" s="35"/>
+      <c r="K37" s="35"/>
+      <c r="L37" s="35"/>
+      <c r="M37" s="36"/>
     </row>
     <row r="38" spans="7:13" ht="15.75" customHeight="1">
-      <c r="G38" s="30"/>
-      <c r="H38" s="31"/>
-      <c r="I38" s="31"/>
-      <c r="J38" s="31"/>
-      <c r="K38" s="31"/>
-      <c r="L38" s="31"/>
-      <c r="M38" s="32"/>
+      <c r="G38" s="37"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="38"/>
+      <c r="J38" s="38"/>
+      <c r="K38" s="38"/>
+      <c r="L38" s="38"/>
+      <c r="M38" s="39"/>
     </row>
     <row r="39" spans="7:13" ht="15.75" customHeight="1"/>
     <row r="40" spans="7:13" ht="15.75" customHeight="1"/>
@@ -2278,26 +2235,25 @@
     <row r="1000" ht="15.75" customHeight="1"/>
     <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="18">
+    <mergeCell ref="G27:M38"/>
+    <mergeCell ref="G23:M23"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="R3:R4"/>
+    <mergeCell ref="O2:R2"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="I3:J4"/>
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="P3:P4"/>
+    <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="B2:J2"/>
     <mergeCell ref="H8:M8"/>
     <mergeCell ref="G20:M20"/>
     <mergeCell ref="G21:M21"/>
     <mergeCell ref="G22:M22"/>
     <mergeCell ref="B8:F8"/>
-    <mergeCell ref="G27:M38"/>
-    <mergeCell ref="G23:M23"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="R3:R4"/>
-    <mergeCell ref="O2:R2"/>
-    <mergeCell ref="B2:M2"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="I3:K3"/>
-    <mergeCell ref="F3:H3"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="L3:M4"/>
-    <mergeCell ref="O3:O4"/>
-    <mergeCell ref="P3:P4"/>
-    <mergeCell ref="Q3:Q4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>